<commit_message>
updated overall progress for S19:Vue3 new: finished Part III
</commit_message>
<xml_diff>
--- a/assets/contents.xlsx
+++ b/assets/contents.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Courses\duyiFe\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Courses\duyiFe\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74B11DB3-9360-4953-A645-E14953843564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B2F3438-FE93-4278-8D75-EE6FCF7E27BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1845" yWindow="1860" windowWidth="21600" windowHeight="11820" tabRatio="722" firstSheet="17" activeTab="20" xr2:uid="{977D219B-3D5A-4B74-BC43-A61DD328A31A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="722" firstSheet="17" activeTab="20" xr2:uid="{977D219B-3D5A-4B74-BC43-A61DD328A31A}"/>
   </bookViews>
   <sheets>
     <sheet name="1HTML_scratch" sheetId="9" r:id="rId1"/>
@@ -42,29 +42,19 @@
     <sheet name="TS_pro" sheetId="29" r:id="rId27"/>
     <sheet name="Echarts" sheetId="20" r:id="rId28"/>
     <sheet name="BPMN" sheetId="22" r:id="rId29"/>
+    <sheet name="Git" sheetId="31" r:id="rId30"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="1204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1419" uniqueCount="1228">
   <si>
     <t>1. 环境准备</t>
   </si>
@@ -3735,6 +3725,88 @@
   </si>
   <si>
     <t>10 11 12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. git的安装和配置</t>
+  </si>
+  <si>
+    <t>2. 暂存和提交</t>
+  </si>
+  <si>
+    <t>3. 分支管理</t>
+  </si>
+  <si>
+    <t>4. 多账号SSH配置规范</t>
+  </si>
+  <si>
+    <t>5. 远程分支的同步</t>
+  </si>
+  <si>
+    <t>6. github flow - 完整流程</t>
+  </si>
+  <si>
+    <t>7. github flow - 协作者和陌生人</t>
+  </si>
+  <si>
+    <t>8. github flow - 冲突变基处理</t>
+  </si>
+  <si>
+    <t>9. github flow - cherry-pick</t>
+  </si>
+  <si>
+    <t>10. github flow - 工作流</t>
+  </si>
+  <si>
+    <t>11. github flow - tag和release</t>
+  </si>
+  <si>
+    <t>12. gitlab flow</t>
+  </si>
+  <si>
+    <t>13. 阿里云效流水线</t>
+  </si>
+  <si>
+    <t>14. worktree</t>
+  </si>
+  <si>
+    <t>备注</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>computed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>学习imooc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>5 7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10 11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>element-plus/ant-design-vue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>14 15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>整理笔记</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>19 20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>20 21</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3742,8 +3814,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="176" formatCode="hh:mm:ss"/>
+    <numFmt numFmtId="177" formatCode="yy\-mm\-dd\ hh:mm"/>
   </numFmts>
   <fonts count="17" x14ac:knownFonts="1">
     <font>
@@ -3809,6 +3882,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -3857,6 +3931,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -4001,7 +4076,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4284,10 +4359,22 @@
     <xf numFmtId="46" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="21" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="46" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -11517,13 +11604,14 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A6EF9A4-06A0-4B42-AB44-860D68BC6616}">
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="47.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="19.5" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>35</v>
       </c>
@@ -11539,17 +11627,24 @@
       <c r="E1" s="94" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="31" t="s">
+      <c r="F1" s="94" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1" s="31" t="s">
         <v>864</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="25" t="s">
         <v>764</v>
       </c>
+      <c r="C2" s="96">
+        <f>SUM(D3:D4)</f>
+        <v>1.983796296296296E-2</v>
+      </c>
       <c r="E2" s="45"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="63" t="s">
         <v>765</v>
       </c>
@@ -11560,14 +11655,17 @@
         <v>10</v>
       </c>
       <c r="D3" s="95">
-        <f t="shared" ref="D3:D34" si="0">B3/1440+C3/86400</f>
+        <f t="shared" ref="D3:D66" si="0">B3/1440+C3/86400</f>
         <v>9.1435185185185178E-3</v>
       </c>
       <c r="E3" s="45">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" s="97">
+        <v>45400.447916666664</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="57" t="s">
         <v>766</v>
       </c>
@@ -11584,886 +11682,1177 @@
       <c r="E4" s="45">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" s="97">
+        <v>45400.467361111114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="s">
         <v>767</v>
       </c>
-      <c r="D5" s="93">
-        <f>SUM(D3:D4)</f>
-        <v>1.983796296296296E-2</v>
+      <c r="C5" s="93">
+        <f>SUM(D6:D35)</f>
+        <v>0.7979166666666665</v>
       </c>
       <c r="E5" s="45"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="G5" s="97"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="63" t="s">
         <v>768</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="57">
         <v>21</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="57">
         <v>27</v>
       </c>
-      <c r="D6" s="91">
+      <c r="D6" s="95">
         <f t="shared" si="0"/>
         <v>1.4895833333333334E-2</v>
       </c>
-      <c r="E6" s="45"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="36" t="s">
+      <c r="E6" s="45">
+        <v>1</v>
+      </c>
+      <c r="G6" s="97">
+        <v>45401.628472222219</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="89" t="s">
         <v>769</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="57">
         <v>33</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="57">
         <v>25</v>
       </c>
-      <c r="D7" s="91">
+      <c r="D7" s="95">
         <f t="shared" si="0"/>
         <v>2.3206018518518518E-2</v>
       </c>
-      <c r="E7" s="45"/>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="36" t="s">
+      <c r="E7" s="45">
+        <v>1</v>
+      </c>
+      <c r="G7" s="97">
+        <v>45401.431944444441</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="89" t="s">
         <v>770</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="57">
         <v>40</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="57">
         <v>25</v>
       </c>
-      <c r="D8" s="91">
+      <c r="D8" s="95">
         <f t="shared" si="0"/>
         <v>2.8067129629629629E-2</v>
       </c>
-      <c r="E8" s="45"/>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="36" t="s">
+      <c r="E8" s="45">
+        <v>2</v>
+      </c>
+      <c r="G8" s="97">
+        <v>45401.472222222219</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="89" t="s">
         <v>771</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="57">
         <v>31</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="57">
         <v>39</v>
       </c>
-      <c r="D9" s="91">
+      <c r="D9" s="95">
         <f t="shared" si="0"/>
         <v>2.1979166666666668E-2</v>
       </c>
-      <c r="E9" s="45"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="E9" s="45">
+        <v>2</v>
+      </c>
+      <c r="F9" t="s">
+        <v>1182</v>
+      </c>
+      <c r="G9" s="97">
+        <v>45401.576388888891</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="57" t="s">
         <v>772</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="57">
         <v>50</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="57">
         <v>19</v>
       </c>
-      <c r="D10" s="91">
+      <c r="D10" s="95">
         <f t="shared" si="0"/>
         <v>3.4942129629629629E-2</v>
       </c>
-      <c r="E10" s="45"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="E10" s="45">
+        <v>2</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1182</v>
+      </c>
+      <c r="G10" s="97">
+        <v>45448.522222222222</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="63" t="s">
         <v>773</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="57">
         <v>30</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="57">
         <v>43</v>
       </c>
-      <c r="D11" s="91">
+      <c r="D11" s="95">
         <f t="shared" si="0"/>
         <v>2.1331018518518517E-2</v>
       </c>
-      <c r="E11" s="45"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="E11" s="45">
+        <v>2</v>
+      </c>
+      <c r="G11" s="97">
+        <v>45448.584722222222</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="57" t="s">
         <v>774</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="57">
         <v>47</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="57">
         <v>1</v>
       </c>
-      <c r="D12" s="91">
+      <c r="D12" s="95">
         <f t="shared" si="0"/>
         <v>3.2650462962962964E-2</v>
       </c>
-      <c r="E12" s="45"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="E12" s="45">
+        <v>2</v>
+      </c>
+      <c r="G12" s="97">
+        <v>45404.6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="57" t="s">
         <v>775</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="57">
         <v>34</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="57">
         <v>9</v>
       </c>
-      <c r="D13" s="91">
+      <c r="D13" s="95">
         <f t="shared" si="0"/>
         <v>2.3715277777777776E-2</v>
       </c>
-      <c r="E13" s="45"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="E13" s="45">
+        <v>2</v>
+      </c>
+      <c r="G13" s="97">
+        <v>45405.379166666666</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="63" t="s">
         <v>776</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="57">
         <v>46</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="57">
         <v>49</v>
       </c>
-      <c r="D14" s="91">
+      <c r="D14" s="95">
         <f t="shared" si="0"/>
         <v>3.2511574074074075E-2</v>
       </c>
-      <c r="E14" s="45"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="E14" s="45">
+        <v>3</v>
+      </c>
+      <c r="G14" s="97">
+        <v>45405.421527777777</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="57" t="s">
         <v>777</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="57">
         <v>41</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="57">
         <v>11</v>
       </c>
-      <c r="D15" s="91">
+      <c r="D15" s="95">
         <f t="shared" si="0"/>
         <v>2.8599537037037038E-2</v>
       </c>
-      <c r="E15" s="45"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="E15" s="45">
+        <v>3</v>
+      </c>
+      <c r="G15" s="97">
+        <v>45405.581944444442</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="63" t="s">
         <v>778</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="57">
         <v>50</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="57">
         <v>4</v>
       </c>
-      <c r="D16" s="91">
+      <c r="D16" s="95">
         <f t="shared" si="0"/>
         <v>3.4768518518518518E-2</v>
       </c>
-      <c r="E16" s="45"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="E16" s="45">
+        <v>3</v>
+      </c>
+      <c r="F16" s="90"/>
+      <c r="G16" s="97">
+        <v>45405.662499999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="57" t="s">
         <v>779</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="57">
         <v>34</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="57">
         <v>20</v>
       </c>
-      <c r="D17" s="91">
+      <c r="D17" s="95">
         <f t="shared" si="0"/>
         <v>2.3842592592592592E-2</v>
       </c>
-      <c r="E17" s="45"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="E17" s="45">
+        <v>3</v>
+      </c>
+      <c r="F17" t="s">
+        <v>1219</v>
+      </c>
+      <c r="G17" s="97">
+        <v>45405.933333333334</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="63" t="s">
         <v>780</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="57">
         <v>32</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="57">
         <v>57</v>
       </c>
-      <c r="D18" s="91">
+      <c r="D18" s="95">
         <f t="shared" si="0"/>
         <v>2.2881944444444444E-2</v>
       </c>
-      <c r="E18" s="45"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="E18" s="45">
+        <v>4</v>
+      </c>
+      <c r="G18" s="97">
+        <v>45406.463194444441</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="63" t="s">
         <v>781</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="57">
         <v>54</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="57">
         <v>37</v>
       </c>
-      <c r="D19" s="91">
+      <c r="D19" s="95">
         <f t="shared" si="0"/>
         <v>3.7928240740740742E-2</v>
       </c>
-      <c r="E19" s="45"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="E19" s="45">
+        <v>4</v>
+      </c>
+      <c r="G19" s="97">
+        <v>45406.555555555555</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="57" t="s">
         <v>782</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="57">
         <v>33</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="57">
         <v>21</v>
       </c>
-      <c r="D20" s="91">
+      <c r="D20" s="95">
         <f t="shared" si="0"/>
         <v>2.315972222222222E-2</v>
       </c>
-      <c r="E20" s="45"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="E20" s="45">
+        <v>4</v>
+      </c>
+      <c r="G20" s="97">
+        <v>45407.432638888888</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="63" t="s">
         <v>783</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="57">
         <v>30</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="57">
         <v>24</v>
       </c>
-      <c r="D21" s="91">
+      <c r="D21" s="95">
         <f t="shared" si="0"/>
         <v>2.1111111111111108E-2</v>
       </c>
-      <c r="E21" s="45"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="E21" s="45">
+        <v>5</v>
+      </c>
+      <c r="F21" t="s">
+        <v>1220</v>
+      </c>
+      <c r="G21" s="97">
+        <v>45407.474999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="57" t="s">
         <v>784</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="57">
         <v>31</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="57">
         <v>48</v>
       </c>
-      <c r="D22" s="91">
+      <c r="D22" s="95">
         <f t="shared" si="0"/>
         <v>2.2083333333333333E-2</v>
       </c>
-      <c r="E22" s="45"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="E22" s="45">
+        <v>5</v>
+      </c>
+      <c r="G22" s="97">
+        <v>45407.572222222225</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="57" t="s">
         <v>785</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="57">
         <v>40</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="57">
         <v>3</v>
       </c>
-      <c r="D23" s="91">
+      <c r="D23" s="95">
         <f t="shared" si="0"/>
         <v>2.7812499999999997E-2</v>
       </c>
-      <c r="E23" s="45"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="E23" s="45" t="s">
+        <v>1221</v>
+      </c>
+      <c r="G23" s="97">
+        <v>45448.629166666666</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="57" t="s">
         <v>786</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="57">
         <v>43</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="57">
         <v>26</v>
       </c>
-      <c r="D24" s="91">
+      <c r="D24" s="95">
         <f t="shared" si="0"/>
         <v>3.0162037037037039E-2</v>
       </c>
-      <c r="E24" s="45"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="E24" s="45" t="s">
+        <v>1197</v>
+      </c>
+      <c r="G24" s="97">
+        <v>45408.455555555556</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="63" t="s">
         <v>787</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="57">
         <v>33</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="57">
         <v>10</v>
       </c>
-      <c r="D25" s="91">
+      <c r="D25" s="95">
         <f t="shared" si="0"/>
         <v>2.3032407407407404E-2</v>
       </c>
-      <c r="E25" s="45"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="E25" s="45">
+        <v>7</v>
+      </c>
+      <c r="G25" s="97">
+        <v>45408.604861111111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="57" t="s">
         <v>788</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="57">
         <v>33</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="57">
         <v>37</v>
       </c>
-      <c r="D26" s="91">
+      <c r="D26" s="95">
         <f t="shared" si="0"/>
         <v>2.3344907407407404E-2</v>
       </c>
-      <c r="E26" s="45"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="E26" s="45">
+        <v>7</v>
+      </c>
+      <c r="G26" s="97">
+        <v>45409.396527777775</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="63" t="s">
         <v>789</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="57">
         <v>42</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="57">
         <v>44</v>
       </c>
-      <c r="D27" s="91">
+      <c r="D27" s="95">
         <f t="shared" si="0"/>
         <v>2.9675925925925925E-2</v>
       </c>
-      <c r="E27" s="45"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="E27" s="45">
+        <v>7</v>
+      </c>
+      <c r="G27" s="97">
+        <v>45409.893750000003</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="57" t="s">
         <v>790</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="57">
         <v>24</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="57">
         <v>28</v>
       </c>
-      <c r="D28" s="91">
+      <c r="D28" s="95">
         <f t="shared" si="0"/>
         <v>1.699074074074074E-2</v>
       </c>
-      <c r="E28" s="45"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="E28" s="45" t="s">
+        <v>1186</v>
+      </c>
+      <c r="G28" s="97">
+        <v>45449.672222222223</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="57" t="s">
         <v>791</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="57">
         <v>35</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="57">
         <v>42</v>
       </c>
-      <c r="D29" s="91">
+      <c r="D29" s="95">
         <f t="shared" si="0"/>
         <v>2.4791666666666667E-2</v>
       </c>
-      <c r="E29" s="45"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="E29" s="45" t="s">
+        <v>1186</v>
+      </c>
+      <c r="G29" s="97">
+        <v>45410.359722222223</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="63" t="s">
         <v>792</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="63">
         <v>43</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="63">
         <v>52</v>
       </c>
-      <c r="D30" s="91">
+      <c r="D30" s="95">
         <f t="shared" si="0"/>
         <v>3.0462962962962966E-2</v>
       </c>
-      <c r="E30" s="45"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="E30" s="45" t="s">
+        <v>1187</v>
+      </c>
+      <c r="G30" s="97">
+        <v>45452.272916666669</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="63" t="s">
         <v>793</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="63">
         <v>48</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="63">
         <v>6</v>
       </c>
-      <c r="D31" s="91">
+      <c r="D31" s="95">
         <f t="shared" si="0"/>
         <v>3.3402777777777774E-2</v>
       </c>
-      <c r="E31" s="45"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="E31" s="45">
+        <v>9</v>
+      </c>
+      <c r="G31" s="97">
+        <v>45452.367361111108</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="63" t="s">
         <v>794</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="63">
         <v>30</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="63">
         <v>9</v>
       </c>
-      <c r="D32" s="91">
+      <c r="D32" s="95">
         <f t="shared" si="0"/>
         <v>2.0937499999999998E-2</v>
       </c>
-      <c r="E32" s="45"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="E32" s="45">
+        <v>10</v>
+      </c>
+      <c r="G32" s="97">
+        <v>45439.628472222219</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="63" t="s">
         <v>795</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="63">
         <v>26</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="63">
         <v>27</v>
       </c>
-      <c r="D33" s="91">
+      <c r="D33" s="95">
         <f t="shared" si="0"/>
         <v>1.8368055555555554E-2</v>
       </c>
-      <c r="E33" s="45"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="E33" s="45">
+        <v>10</v>
+      </c>
+      <c r="G33" s="97">
+        <v>45452.948611111111</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="63" t="s">
         <v>796</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="63">
         <v>39</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="63">
         <v>54</v>
       </c>
-      <c r="D34" s="91">
+      <c r="D34" s="95">
         <f t="shared" si="0"/>
         <v>2.7708333333333335E-2</v>
       </c>
-      <c r="E34" s="45"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="E34" s="45" t="s">
+        <v>1222</v>
+      </c>
+      <c r="G34" s="97">
+        <v>45453.760416666664</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" s="63" t="s">
         <v>797</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="57">
         <v>62</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="57">
         <v>43</v>
       </c>
-      <c r="D35" s="91">
-        <f t="shared" ref="D35:D66" si="1">B35/1440+C35/86400</f>
+      <c r="D35" s="95">
+        <f t="shared" si="0"/>
         <v>4.355324074074074E-2</v>
       </c>
-      <c r="E35" s="45"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E35" s="45" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1223</v>
+      </c>
+      <c r="G35" s="97">
+        <v>45453.861805555556</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="25" t="s">
         <v>798</v>
       </c>
-      <c r="D36" s="93">
-        <f>SUM(D6:D35)</f>
-        <v>0.7979166666666665</v>
+      <c r="C36" s="93">
+        <f>SUM(D37:D58)</f>
+        <v>0.65162037037037013</v>
       </c>
       <c r="E36" s="45"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="63" t="s">
         <v>799</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="57">
         <v>18</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="57">
         <v>22</v>
       </c>
-      <c r="D37" s="91">
-        <f t="shared" si="1"/>
+      <c r="D37" s="95">
+        <f t="shared" si="0"/>
         <v>1.275462962962963E-2</v>
       </c>
-      <c r="E37" s="45"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+      <c r="E37" s="45">
+        <v>13</v>
+      </c>
+      <c r="G37" s="97">
+        <v>45433.911805555559</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" s="57" t="s">
         <v>800</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="57">
         <v>87</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="57">
         <v>40</v>
       </c>
-      <c r="D38" s="91">
-        <f t="shared" si="1"/>
+      <c r="D38" s="95">
+        <f t="shared" si="0"/>
         <v>6.0879629629629631E-2</v>
       </c>
-      <c r="E38" s="45"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="E38" s="45">
+        <v>13</v>
+      </c>
+      <c r="G38" s="97">
+        <v>45421.581944444442</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="57" t="s">
         <v>801</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="57">
         <v>59</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="57">
         <v>4</v>
       </c>
-      <c r="D39" s="91">
-        <f t="shared" si="1"/>
+      <c r="D39" s="95">
+        <f t="shared" si="0"/>
         <v>4.1018518518518517E-2</v>
       </c>
-      <c r="E39" s="45"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="E39" s="45">
+        <v>13</v>
+      </c>
+      <c r="G39" s="97">
+        <v>45422.586111111108</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="63" t="s">
         <v>802</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="57">
         <v>24</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="57">
         <v>5</v>
       </c>
-      <c r="D40" s="91">
-        <f t="shared" si="1"/>
+      <c r="D40" s="95">
+        <f t="shared" si="0"/>
         <v>1.6724537037037038E-2</v>
       </c>
-      <c r="E40" s="45"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="E40" s="45">
+        <v>14</v>
+      </c>
+      <c r="G40" s="97">
+        <v>45432.881944444445</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" s="57" t="s">
         <v>803</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="57">
         <v>59</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="57">
         <v>53</v>
       </c>
-      <c r="D41" s="91">
-        <f t="shared" si="1"/>
+      <c r="D41" s="95">
+        <f t="shared" si="0"/>
         <v>4.1585648148148149E-2</v>
       </c>
-      <c r="E41" s="45"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+      <c r="E41" s="45" t="s">
+        <v>1224</v>
+      </c>
+      <c r="F41" t="s">
+        <v>1225</v>
+      </c>
+      <c r="G41" s="97">
+        <v>45434.326388888891</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="57" t="s">
         <v>804</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="57">
         <v>52</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="57">
         <v>12</v>
       </c>
-      <c r="D42" s="91">
-        <f t="shared" si="1"/>
+      <c r="D42" s="95">
+        <f t="shared" si="0"/>
         <v>3.6249999999999998E-2</v>
       </c>
-      <c r="E42" s="45"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="E42" s="45" t="s">
+        <v>1224</v>
+      </c>
+      <c r="F42" t="s">
+        <v>1225</v>
+      </c>
+      <c r="G42" s="97">
+        <v>45434.534722222219</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="63" t="s">
         <v>805</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="57">
         <v>53</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="57">
         <v>11</v>
       </c>
-      <c r="D43" s="91">
-        <f t="shared" si="1"/>
+      <c r="D43" s="95">
+        <f t="shared" si="0"/>
         <v>3.6932870370370373E-2</v>
       </c>
-      <c r="E43" s="45"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="E43" s="45">
+        <v>16</v>
+      </c>
+      <c r="G43" s="97">
+        <v>45435.498611111114</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="63" t="s">
         <v>806</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="57">
         <v>40</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="57">
         <v>55</v>
       </c>
-      <c r="D44" s="91">
-        <f t="shared" si="1"/>
+      <c r="D44" s="95">
+        <f t="shared" si="0"/>
         <v>2.841435185185185E-2</v>
       </c>
-      <c r="E44" s="45"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="E44" s="45">
+        <v>16</v>
+      </c>
+      <c r="G44" s="97">
+        <v>45436.490972222222</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" s="63" t="s">
         <v>807</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="57">
         <v>55</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="57">
         <v>6</v>
       </c>
-      <c r="D45" s="91">
-        <f t="shared" si="1"/>
+      <c r="D45" s="95">
+        <f t="shared" si="0"/>
         <v>3.8263888888888889E-2</v>
       </c>
-      <c r="E45" s="45"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="E45" s="45">
+        <v>16</v>
+      </c>
+      <c r="G45" s="98">
+        <v>45445.297222222223</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="63" t="s">
         <v>808</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="57">
         <v>44</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="57">
         <v>32</v>
       </c>
-      <c r="D46" s="91">
-        <f t="shared" si="1"/>
+      <c r="D46" s="95">
+        <f t="shared" si="0"/>
         <v>3.0925925925925926E-2</v>
       </c>
-      <c r="E46" s="45"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="E46" s="45">
+        <v>17</v>
+      </c>
+      <c r="G46" s="98">
+        <v>45446.452777777777</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="57" t="s">
         <v>809</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="57">
         <v>50</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="57">
         <v>42</v>
       </c>
-      <c r="D47" s="91">
-        <f t="shared" si="1"/>
+      <c r="D47" s="95">
+        <f t="shared" si="0"/>
         <v>3.5208333333333335E-2</v>
       </c>
-      <c r="E47" s="45"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+      <c r="E47" s="45">
+        <v>18</v>
+      </c>
+      <c r="G47" s="98">
+        <v>45446.537499999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" s="57" t="s">
         <v>810</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="57">
         <v>49</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="57">
         <v>2</v>
       </c>
-      <c r="D48" s="91">
-        <f t="shared" si="1"/>
+      <c r="D48" s="95">
+        <f t="shared" si="0"/>
         <v>3.4050925925925922E-2</v>
       </c>
-      <c r="E48" s="45"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+      <c r="E48" s="45">
+        <v>18</v>
+      </c>
+      <c r="G48" s="98">
+        <v>45446.591666666667</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="57" t="s">
         <v>811</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="57">
         <v>26</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="57">
         <v>38</v>
       </c>
-      <c r="D49" s="91">
-        <f t="shared" si="1"/>
+      <c r="D49" s="95">
+        <f t="shared" si="0"/>
         <v>1.849537037037037E-2</v>
       </c>
-      <c r="E49" s="45"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+      <c r="E49" s="45">
+        <v>19</v>
+      </c>
+      <c r="G49" s="98">
+        <v>45446.90902777778</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" s="63" t="s">
         <v>812</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="57">
         <v>25</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="57">
         <v>1</v>
       </c>
-      <c r="D50" s="91">
-        <f t="shared" si="1"/>
+      <c r="D50" s="95">
+        <f t="shared" si="0"/>
         <v>1.7372685185185185E-2</v>
       </c>
-      <c r="E50" s="45"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="E50" s="45">
+        <v>19</v>
+      </c>
+      <c r="G50" s="98">
+        <v>45446.938194444447</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" s="57" t="s">
         <v>813</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="57">
         <v>18</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="57">
         <v>13</v>
       </c>
-      <c r="D51" s="91">
-        <f t="shared" si="1"/>
+      <c r="D51" s="95">
+        <f t="shared" si="0"/>
         <v>1.2650462962962964E-2</v>
       </c>
-      <c r="E51" s="45"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+      <c r="E51" s="45">
+        <v>19</v>
+      </c>
+      <c r="G51" s="97">
+        <v>45439.459027777775</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" s="63" t="s">
         <v>814</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="57">
         <v>32</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="57">
         <v>5</v>
       </c>
-      <c r="D52" s="91">
-        <f t="shared" si="1"/>
+      <c r="D52" s="95">
+        <f t="shared" si="0"/>
         <v>2.2280092592592594E-2</v>
       </c>
-      <c r="E52" s="45"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+      <c r="E52" s="45" t="s">
+        <v>1226</v>
+      </c>
+      <c r="G52" s="97">
+        <v>45435.586111111108</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" s="57" t="s">
         <v>815</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="57">
         <v>36</v>
       </c>
-      <c r="C53">
+      <c r="C53" s="57">
         <v>58</v>
       </c>
-      <c r="D53" s="91">
-        <f t="shared" si="1"/>
+      <c r="D53" s="95">
+        <f t="shared" si="0"/>
         <v>2.5671296296296296E-2</v>
       </c>
-      <c r="E53" s="45"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+      <c r="E53" s="45" t="s">
+        <v>1226</v>
+      </c>
+      <c r="G53" s="97">
+        <v>45439.522916666669</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" s="57" t="s">
         <v>816</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="57">
         <v>62</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="57">
         <v>44</v>
       </c>
-      <c r="D54" s="91">
-        <f t="shared" si="1"/>
+      <c r="D54" s="95">
+        <f t="shared" si="0"/>
         <v>4.3564814814814813E-2</v>
       </c>
-      <c r="E54" s="45"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+      <c r="E54" s="45" t="s">
+        <v>1226</v>
+      </c>
+      <c r="G54" s="97">
+        <v>45435.910416666666</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" s="57" t="s">
         <v>817</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="57">
         <v>38</v>
       </c>
-      <c r="C55">
+      <c r="C55" s="57">
         <v>17</v>
       </c>
-      <c r="D55" s="91">
-        <f t="shared" si="1"/>
+      <c r="D55" s="95">
+        <f t="shared" si="0"/>
         <v>2.6585648148148146E-2</v>
       </c>
-      <c r="E55" s="45"/>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+      <c r="E55" s="45">
+        <v>20</v>
+      </c>
+      <c r="G55" s="97">
+        <v>45440.898611111108</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" s="57" t="s">
         <v>818</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="57">
         <v>25</v>
       </c>
-      <c r="C56">
+      <c r="C56" s="57">
         <v>47</v>
       </c>
-      <c r="D56" s="91">
-        <f t="shared" si="1"/>
+      <c r="D56" s="95">
+        <f t="shared" si="0"/>
         <v>1.7905092592592594E-2</v>
       </c>
-      <c r="E56" s="45"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+      <c r="E56" s="45" t="s">
+        <v>1227</v>
+      </c>
+      <c r="G56" s="97">
+        <v>45441.93472222222</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" s="63" t="s">
         <v>819</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="57">
         <v>33</v>
       </c>
-      <c r="C57">
+      <c r="C57" s="57">
         <v>17</v>
       </c>
-      <c r="D57" s="91">
-        <f t="shared" si="1"/>
+      <c r="D57" s="95">
+        <f t="shared" si="0"/>
         <v>2.3113425925925923E-2</v>
       </c>
-      <c r="E57" s="45"/>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+      <c r="E57" s="45">
+        <v>21</v>
+      </c>
+      <c r="G57" s="97">
+        <v>45444.939583333333</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" s="57" t="s">
         <v>820</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="57">
         <v>44</v>
       </c>
-      <c r="C58">
+      <c r="C58" s="57">
         <v>36</v>
       </c>
-      <c r="D58" s="91">
-        <f t="shared" si="1"/>
+      <c r="D58" s="95">
+        <f t="shared" si="0"/>
         <v>3.097222222222222E-2</v>
       </c>
-      <c r="E58" s="45"/>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E58" s="45">
+        <v>21</v>
+      </c>
+      <c r="G58" s="97">
+        <v>45439.416666666664</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" s="25" t="s">
         <v>821</v>
       </c>
-      <c r="D59" s="93">
-        <f>SUM(D37:D58)</f>
-        <v>0.65162037037037013</v>
+      <c r="C59" s="93">
+        <f>SUM(D60:D102)</f>
+        <v>1.0073379629629633</v>
       </c>
       <c r="E59" s="45"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" s="57" t="s">
         <v>799</v>
       </c>
-      <c r="B60">
+      <c r="B60" s="57">
         <v>6</v>
       </c>
-      <c r="C60">
+      <c r="C60" s="57">
         <v>9</v>
       </c>
-      <c r="D60" s="91">
-        <f t="shared" si="1"/>
+      <c r="D60" s="95">
+        <f t="shared" si="0"/>
         <v>4.2708333333333331E-3</v>
       </c>
-      <c r="E60" s="45"/>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E60" s="45">
+        <v>21</v>
+      </c>
+      <c r="G60" s="99">
+        <v>45502.651388888888</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>822</v>
       </c>
@@ -12474,12 +12863,12 @@
         <v>36</v>
       </c>
       <c r="D61" s="91">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.2916666666666667E-2</v>
       </c>
       <c r="E61" s="45"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>823</v>
       </c>
@@ -12490,12 +12879,12 @@
         <v>54</v>
       </c>
       <c r="D62" s="91">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.2152777777777778E-2</v>
       </c>
       <c r="E62" s="45"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>824</v>
       </c>
@@ -12506,12 +12895,12 @@
         <v>2</v>
       </c>
       <c r="D63" s="91">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.7106481481481481E-2</v>
       </c>
       <c r="E63" s="45"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>825</v>
       </c>
@@ -12522,7 +12911,7 @@
         <v>51</v>
       </c>
       <c r="D64" s="91">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.6979166666666665E-2</v>
       </c>
       <c r="E64" s="45"/>
@@ -12538,7 +12927,7 @@
         <v>8</v>
       </c>
       <c r="D65" s="91">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.6481481481481481E-2</v>
       </c>
       <c r="E65" s="45"/>
@@ -12554,7 +12943,7 @@
         <v>2</v>
       </c>
       <c r="D66" s="91">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.5856481481481477E-2</v>
       </c>
       <c r="E66" s="45"/>
@@ -12570,7 +12959,7 @@
         <v>59</v>
       </c>
       <c r="D67" s="91">
-        <f t="shared" ref="D67:D98" si="2">B67/1440+C67/86400</f>
+        <f t="shared" ref="D67:D102" si="1">B67/1440+C67/86400</f>
         <v>1.7349537037037038E-2</v>
       </c>
       <c r="E67" s="45"/>
@@ -12586,7 +12975,7 @@
         <v>44</v>
       </c>
       <c r="D68" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.1620370370370371E-2</v>
       </c>
       <c r="E68" s="45"/>
@@ -12602,7 +12991,7 @@
         <v>1</v>
       </c>
       <c r="D69" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.1817129629629629E-2</v>
       </c>
       <c r="E69" s="45"/>
@@ -12618,7 +13007,7 @@
         <v>36</v>
       </c>
       <c r="D70" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.7083333333333332E-2</v>
       </c>
       <c r="E70" s="45"/>
@@ -12634,7 +13023,7 @@
         <v>34</v>
       </c>
       <c r="D71" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.1921296296296296E-2</v>
       </c>
       <c r="E71" s="45"/>
@@ -12650,7 +13039,7 @@
         <v>59</v>
       </c>
       <c r="D72" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.5266203703703704E-2</v>
       </c>
       <c r="E72" s="45"/>
@@ -12666,7 +13055,7 @@
         <v>49</v>
       </c>
       <c r="D73" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.5150462962962963E-2</v>
       </c>
       <c r="E73" s="45"/>
@@ -12682,7 +13071,7 @@
         <v>28</v>
       </c>
       <c r="D74" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.4212962962962962E-2</v>
       </c>
       <c r="E74" s="45"/>
@@ -12698,7 +13087,7 @@
         <v>20</v>
       </c>
       <c r="D75" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.0370370370370372E-2</v>
       </c>
       <c r="E75" s="45"/>
@@ -12714,7 +13103,7 @@
         <v>16</v>
       </c>
       <c r="D76" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.2546296296296297E-2</v>
       </c>
       <c r="E76" s="45"/>
@@ -12730,7 +13119,7 @@
         <v>17</v>
       </c>
       <c r="D77" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.4780092592592593E-2</v>
       </c>
       <c r="E77" s="45"/>
@@ -12746,7 +13135,7 @@
         <v>35</v>
       </c>
       <c r="D78" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.3599537037037037E-2</v>
       </c>
       <c r="E78" s="45"/>
@@ -12762,7 +13151,7 @@
         <v>42</v>
       </c>
       <c r="D79" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.7708333333333332E-2</v>
       </c>
       <c r="E79" s="45"/>
@@ -12778,7 +13167,7 @@
         <v>36</v>
       </c>
       <c r="D80" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.4444444444444444E-2</v>
       </c>
       <c r="E80" s="45"/>
@@ -12794,7 +13183,7 @@
         <v>12</v>
       </c>
       <c r="D81" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.027777777777778E-2</v>
       </c>
       <c r="E81" s="45"/>
@@ -12810,7 +13199,7 @@
         <v>24</v>
       </c>
       <c r="D82" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.9861111111111111E-2</v>
       </c>
       <c r="E82" s="45"/>
@@ -12826,7 +13215,7 @@
         <v>33</v>
       </c>
       <c r="D83" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.4270833333333333E-2</v>
       </c>
       <c r="E83" s="45"/>
@@ -12842,7 +13231,7 @@
         <v>23</v>
       </c>
       <c r="D84" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.9849537037037037E-2</v>
       </c>
       <c r="E84" s="45"/>
@@ -12858,7 +13247,7 @@
         <v>53</v>
       </c>
       <c r="D85" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.1585648148148149E-2</v>
       </c>
       <c r="E85" s="45"/>
@@ -12874,7 +13263,7 @@
         <v>52</v>
       </c>
       <c r="D86" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.740740740740741E-2</v>
       </c>
       <c r="E86" s="45"/>
@@ -12890,7 +13279,7 @@
         <v>7</v>
       </c>
       <c r="D87" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.0914351851851851E-2</v>
       </c>
       <c r="E87" s="45"/>
@@ -12906,7 +13295,7 @@
         <v>21</v>
       </c>
       <c r="D88" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.1354166666666667E-2</v>
       </c>
       <c r="E88" s="45"/>
@@ -12922,7 +13311,7 @@
         <v>32</v>
       </c>
       <c r="D89" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.1481481481481481E-2</v>
       </c>
       <c r="E89" s="45"/>
@@ -12938,7 +13327,7 @@
         <v>51</v>
       </c>
       <c r="D90" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.8090277777777778E-2</v>
       </c>
       <c r="E90" s="45"/>
@@ -12954,7 +13343,7 @@
         <v>54</v>
       </c>
       <c r="D91" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.6597222222222222E-2</v>
       </c>
       <c r="E91" s="45"/>
@@ -12970,7 +13359,7 @@
         <v>6</v>
       </c>
       <c r="D92" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.0624999999999999E-2</v>
       </c>
       <c r="E92" s="45"/>
@@ -12986,7 +13375,7 @@
         <v>30</v>
       </c>
       <c r="D93" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.8402777777777775E-2</v>
       </c>
       <c r="E93" s="45"/>
@@ -13002,7 +13391,7 @@
         <v>17</v>
       </c>
       <c r="D94" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.4641203703703704E-2</v>
       </c>
       <c r="E94" s="45"/>
@@ -13018,7 +13407,7 @@
         <v>22</v>
       </c>
       <c r="D95" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.8310185185185183E-2</v>
       </c>
       <c r="E95" s="45"/>
@@ -13034,7 +13423,7 @@
         <v>10</v>
       </c>
       <c r="D96" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.0671296296296294E-2</v>
       </c>
       <c r="E96" s="45"/>
@@ -13050,7 +13439,7 @@
         <v>43</v>
       </c>
       <c r="D97" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.1331018518518517E-2</v>
       </c>
       <c r="E97" s="45"/>
@@ -13066,7 +13455,7 @@
         <v>16</v>
       </c>
       <c r="D98" s="91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.2129629629629626E-2</v>
       </c>
       <c r="E98" s="45"/>
@@ -13082,7 +13471,7 @@
         <v>24</v>
       </c>
       <c r="D99" s="91">
-        <f t="shared" ref="D99:D102" si="3">B99/1440+C99/86400</f>
+        <f t="shared" si="1"/>
         <v>1.5555555555555555E-2</v>
       </c>
       <c r="E99" s="45"/>
@@ -13098,7 +13487,7 @@
         <v>42</v>
       </c>
       <c r="D100" s="91">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>2.4097222222222221E-2</v>
       </c>
       <c r="E100" s="45"/>
@@ -13114,7 +13503,7 @@
         <v>30</v>
       </c>
       <c r="D101" s="91">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>1.2847222222222223E-2</v>
       </c>
       <c r="E101" s="45"/>
@@ -13130,7 +13519,7 @@
         <v>54</v>
       </c>
       <c r="D102" s="91">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>3.402777777777778E-3</v>
       </c>
       <c r="E102" s="45"/>
@@ -13138,16 +13527,43 @@
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" s="11" t="str">
         <f>"总时长："&amp;TEXT(SUM(B:B)/1440+SUM(C:C)/86400,"[h]:mm:ss")</f>
-        <v>总时长：59:26:28</v>
-      </c>
-      <c r="D103" s="93">
-        <f>SUM(D60:D102)</f>
-        <v>1.0073379629629633</v>
+        <v>总时长：59:26:30</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="D60:D102">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{8275B0C3-DF87-4C89-9CAC-283E048F50B2}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{8275B0C3-DF87-4C89-9CAC-283E048F50B2}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D60:D102</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -18432,6 +18848,198 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CEFC2E3-EED2-454A-8E0C-28D2F8839966}">
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="45" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.2">
+      <c r="A1" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="79" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B2">
+        <v>24</v>
+      </c>
+      <c r="C2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>1205</v>
+      </c>
+      <c r="B3">
+        <v>25</v>
+      </c>
+      <c r="C3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B4">
+        <v>33</v>
+      </c>
+      <c r="C4">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>1207</v>
+      </c>
+      <c r="B5">
+        <v>25</v>
+      </c>
+      <c r="C5">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>1208</v>
+      </c>
+      <c r="B6">
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+      <c r="C7">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B8">
+        <v>24</v>
+      </c>
+      <c r="C8">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B9">
+        <v>19</v>
+      </c>
+      <c r="C9">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>1212</v>
+      </c>
+      <c r="B10">
+        <v>12</v>
+      </c>
+      <c r="C10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>1213</v>
+      </c>
+      <c r="B11">
+        <v>39</v>
+      </c>
+      <c r="C11">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>1214</v>
+      </c>
+      <c r="B12">
+        <v>16</v>
+      </c>
+      <c r="C12">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>1215</v>
+      </c>
+      <c r="B13">
+        <v>13</v>
+      </c>
+      <c r="C13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>1216</v>
+      </c>
+      <c r="B14">
+        <v>26</v>
+      </c>
+      <c r="C14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B15">
+        <v>8</v>
+      </c>
+      <c r="C15">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="58" t="str">
+        <f>"总时长："&amp;TEXT(SUM(B:B)/1440+SUM(C:C)/86400,"[h]:mm:ss")</f>
+        <v>总时长：5:30:46</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>